<commit_message>
Fix AI output accuracy - CFO email language, variance truncation, headcount summary
</commit_message>
<xml_diff>
--- a/data/Helvetia_AG_AI_Synthetic_Datasets.xlsx
+++ b/data/Helvetia_AG_AI_Synthetic_Datasets.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suhas\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suhas\Documents\Z11.AIProjects\A1.Month-EndCloseManager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8740B26-F0E9-4696-A789-2D9DF1EEEDD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E83733-96A1-4FD2-9EDC-E736FA2B9729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -747,15 +747,9 @@
     <t>CHF 22K</t>
   </si>
   <si>
-    <t>CHF 148K adverse vs budget</t>
-  </si>
-  <si>
     <t>States 'marginally below budget'</t>
   </si>
   <si>
-    <t>CHF 148K</t>
-  </si>
-  <si>
     <t>Entity</t>
   </si>
   <si>
@@ -976,6 +970,12 @@
   </si>
   <si>
     <t>Note: Monthly cost impact reflects salary-only rates for permanent role movements. Excludes contractor costs (reported separately in Variance Root Cause), bonus accruals, and social charges. Currency conversion to CHF not applied in this dataset.</t>
+  </si>
+  <si>
+    <t>CHF 178K adverse vs budget</t>
+  </si>
+  <si>
+    <t>CHF 178K</t>
   </si>
 </sst>
 </file>
@@ -995,33 +995,39 @@
       <sz val="11"/>
       <color rgb="FF1F4E79"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF1F4E79"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1162,13 +1168,13 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1486,32 +1492,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>271</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="A1" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>272</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
+      <c r="A2" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1699,7 +1705,7 @@
         <v>-28000</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -1825,7 +1831,7 @@
         <v>-25300</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -1889,7 +1895,7 @@
         <v>-13500</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1984,7 +1990,7 @@
         <v>-9000</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -2079,7 +2085,7 @@
         <v>-45000</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2170,34 +2176,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>278</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="A1" s="17" t="s">
+        <v>276</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>279</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="A2" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
     </row>
     <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2453,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2675,7 +2681,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2749,7 +2755,7 @@
         <v>0</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2786,7 +2792,7 @@
         <v>-22000</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2812,30 +2818,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>282</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
+      <c r="A1" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>283</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="A2" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2921,7 +2927,7 @@
         <v>138</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3008,7 +3014,7 @@
         <v>138</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3037,7 +3043,7 @@
         <v>138</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3124,7 +3130,7 @@
         <v>138</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3179,10 +3185,10 @@
         <v>166</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3211,7 +3217,7 @@
         <v>138</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3411,10 +3417,10 @@
         <v>166</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3440,7 +3446,7 @@
         <v>166</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>184</v>
@@ -3472,7 +3478,7 @@
         <v>138</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3659,37 +3665,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
+        <v>291</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>294</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
-        <v>295</v>
-      </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
     </row>
     <row r="4" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -3769,15 +3775,15 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>296</v>
-      </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
+      <c r="A12" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -3833,7 +3839,7 @@
         <v>221</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>222</v>
@@ -3842,7 +3848,7 @@
         <v>223</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>224</v>
@@ -3868,7 +3874,7 @@
         <v>219</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -3914,7 +3920,7 @@
         <v>219</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="87" customHeight="1" x14ac:dyDescent="0.25">
@@ -3925,19 +3931,19 @@
         <v>125</v>
       </c>
       <c r="C19" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>237</v>
-      </c>
       <c r="E19" s="5" t="s">
-        <v>238</v>
+        <v>312</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>219</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -3967,76 +3973,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>300</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="A1" s="17" t="s">
+        <v>298</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>301</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="A2" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
     </row>
     <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C4" s="4">
         <v>42</v>
@@ -4063,15 +4069,15 @@
         <v>55500</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>37</v>
@@ -4100,18 +4106,18 @@
         <v>0</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C6" s="5">
         <v>8</v>
@@ -4138,15 +4144,15 @@
         <v>-12000</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>25</v>
@@ -4175,18 +4181,18 @@
         <v>0</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C8" s="2">
         <v>15</v>
@@ -4212,18 +4218,18 @@
         <v>0</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C9" s="3">
         <v>4</v>
@@ -4249,18 +4255,18 @@
         <v>0</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C10" s="9">
         <v>99</v>
@@ -4289,18 +4295,18 @@
         <v>43500</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C12" s="4">
         <v>38</v>
@@ -4327,15 +4333,15 @@
         <v>48600</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>37</v>
@@ -4365,18 +4371,18 @@
         <v>44400</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C14" s="2">
         <v>9</v>
@@ -4402,15 +4408,15 @@
         <v>0</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>25</v>
@@ -4440,18 +4446,18 @@
         <v>26800</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C16" s="4">
         <v>24</v>
@@ -4478,18 +4484,18 @@
         <v>22400</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C17" s="4">
         <v>3</v>
@@ -4516,18 +4522,18 @@
         <v>15600</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C18" s="9">
         <v>104</v>
@@ -4556,18 +4562,18 @@
         <v>157800</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C20" s="2">
         <v>19</v>
@@ -4593,15 +4599,15 @@
         <v>0</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>37</v>
@@ -4630,18 +4636,18 @@
         <v>0</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C22" s="2">
         <v>5</v>
@@ -4667,15 +4673,15 @@
         <v>0</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -4704,18 +4710,18 @@
         <v>0</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C24" s="2">
         <v>12</v>
@@ -4741,18 +4747,18 @@
         <v>0</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C25" s="9">
         <v>53</v>
@@ -4777,15 +4783,15 @@
         <v>0</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -4800,7 +4806,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B28" s="7">
         <v>256</v>
@@ -4817,7 +4823,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B29" s="7">
         <v>263</v>
@@ -4834,7 +4840,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B30" s="7">
         <v>7</v>
@@ -4851,7 +4857,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B31" s="7">
         <v>7</v>
@@ -4871,7 +4877,7 @@
         <v>68</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
@@ -4884,8 +4890,8 @@
       <c r="K32" s="7"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="20" t="s">
-        <v>312</v>
+      <c r="A33" s="16" t="s">
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>